<commit_message>
Auto update 2026-08-24 08:12:02
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,72 +436,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>51311301g</t>
+          <t>LC47208G-1X</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51311301g/001.jpg,https://oleks-netizen.github.io/product-images/51311301g/002.jpg,https://oleks-netizen.github.io/product-images/51311301g/004.jpg,https://oleks-netizen.github.io/product-images/51311301g/005.jpg,https://oleks-netizen.github.io/product-images/51311301g/006.jpg,https://oleks-netizen.github.io/product-images/51311301g/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47208G-1X/001.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/002.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/003.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/004.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/005.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/006.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/007.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/008.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>51311506g</t>
+          <t>LC47210-93</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/51311506g/001.jpg,https://oleks-netizen.github.io/product-images/51311506g/002.jpg,https://oleks-netizen.github.io/product-images/51311506g/004.jpg,https://oleks-netizen.github.io/product-images/51311506g/005.jpg,https://oleks-netizen.github.io/product-images/51311506g/006.jpg,https://oleks-netizen.github.io/product-images/51311506g/007.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47210-93/001.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/002.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/004.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/005.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/006.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/007.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/008.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/009.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>90321064g</t>
+          <t>LC47541-1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90321064g/001.jpg,https://oleks-netizen.github.io/product-images/90321064g/003.jpg,https://oleks-netizen.github.io/product-images/90321064g/004.jpg,https://oleks-netizen.github.io/product-images/90321064g/005.jpg,https://oleks-netizen.github.io/product-images/90321064g/006.jpg,https://oleks-netizen.github.io/product-images/90321064g/007.jpg,https://oleks-netizen.github.io/product-images/90321064g/008.jpg,https://oleks-netizen.github.io/product-images/90321064g/009.jpg,https://oleks-netizen.github.io/product-images/90321064g/010.jpg,https://oleks-netizen.github.io/product-images/90321064g/011.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47541-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/007.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/008.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/009.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HB2080WHS</t>
+          <t>LC47541-93</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/HB2080WHS/001.jpg,https://oleks-netizen.github.io/product-images/HB2080WHS/002.jpg,https://oleks-netizen.github.io/product-images/HB2080WHS/004.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47541-93/001.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/002.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/004.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/005.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/006.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/007.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/008.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/009.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/010.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LC46022A-1</t>
+          <t>LC47554-1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46022A-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46022A-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47554-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/007.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/008.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -511,12 +511,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LC46026-1</t>
+          <t>LC47632F-1C</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46026-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/003.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46026-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47632F-1C/001.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/002.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/003.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/004.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/005.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/006.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/007.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/008.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -526,12 +526,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LC46026-2</t>
+          <t>LC47832-1C</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46026-2/001.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/003.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/004.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/005.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/006.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/007.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/008.jpg,https://oleks-netizen.github.io/product-images/LC46026-2/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47832-1C/001.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/002.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/003.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/004.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/005.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/006.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/007.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/008.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -541,12 +541,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LC46102-1</t>
+          <t>LC47832-93</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46102-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/003.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46102-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47832-93/001.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/002.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/003.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/004.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/005.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/006.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/007.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/008.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -556,12 +556,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LC46112-1</t>
+          <t>LC47891-1C</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46112-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/003.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46112-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/LC47891-1C/001.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/002.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/003.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/004.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/005.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/006.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/007.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/008.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -571,211 +571,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LC46112-2</t>
+          <t>RJ-hold-3md</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46112-2/001.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/003.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/004.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/005.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/006.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/007.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/008.jpg,https://oleks-netizen.github.io/product-images/LC46112-2/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/RJ-hold-3md/001.jpg,https://oleks-netizen.github.io/product-images/RJ-hold-3md/002.jpg,https://oleks-netizen.github.io/product-images/RJ-hold-3md/003.jpg,https://oleks-netizen.github.io/product-images/RJ-hold-3md/005.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>LC46126-1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46126-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/003.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46126-1/008.jpg</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>LC46127-1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46127-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/003.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46127-1/008.jpg</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>LC46127-2</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46127-2/001.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/002.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/004.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/005.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/006.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/007.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/008.jpg,https://oleks-netizen.github.io/product-images/LC46127-2/009.jpg</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>LC46154B-1</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46154B-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46154B-1/009.jpg</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>LC46154B-2</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46154B-2/001.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/002.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/004.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/005.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/006.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/007.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/008.jpg,https://oleks-netizen.github.io/product-images/LC46154B-2/009.jpg</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>LC46192A-2</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46192A-2/001.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/002.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/004.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/005.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/006.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/007.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/008.jpg,https://oleks-netizen.github.io/product-images/LC46192A-2/009.jpg</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>LC46226-1</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46226-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46226-1/009.jpg</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>LC46226-2</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46226-2/001.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/002.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/004.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/005.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/006.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/007.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/008.jpg,https://oleks-netizen.github.io/product-images/LC46226-2/009.jpg</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>LC46547-1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46547-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46547-1/009.jpg</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>LC46601-1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46601-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46601-1/009.jpg</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>LC46621-1</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46621-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46621-1/009.jpg</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>LC46984-1</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/LC46984-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46984-1/009.jpg</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>RAG-1810-3md</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/RAG-1810-3md/001.jpg,https://oleks-netizen.github.io/product-images/RAG-1810-3md/002.jpg,https://oleks-netizen.github.io/product-images/RAG-1810-3md/004.jpg,https://oleks-netizen.github.io/product-images/RAG-1810-3md/005.jpg,https://oleks-netizen.github.io/product-images/RAG-1810-3md/006.jpg,https://oleks-netizen.github.io/product-images/RAG-1810-3md/007.jpg,https://oleks-netizen.github.io/product-images/RAG-1810-3md/008.jpg</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-08-24 10:24:43
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,42 +436,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LC47208G-1X</t>
+          <t>11711001g</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47208G-1X/001.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/002.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/003.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/004.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/005.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/006.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/007.jpg,https://oleks-netizen.github.io/product-images/LC47208G-1X/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711001g/001.jpg,https://oleks-netizen.github.io/product-images/11711001g/002.jpg,https://oleks-netizen.github.io/product-images/11711001g/003.jpg,https://oleks-netizen.github.io/product-images/11711001g/004.jpg,https://oleks-netizen.github.io/product-images/11711001g/005.jpg,https://oleks-netizen.github.io/product-images/11711001g/006.jpg,https://oleks-netizen.github.io/product-images/11711001g/008.jpg,https://oleks-netizen.github.io/product-images/11711001g/009.jpg,https://oleks-netizen.github.io/product-images/11711001g/010.jpg,https://oleks-netizen.github.io/product-images/11711001g/011.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LC47210-93</t>
+          <t>11711001s</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47210-93/001.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/002.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/004.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/005.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/006.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/007.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/008.jpg,https://oleks-netizen.github.io/product-images/LC47210-93/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711001s/001.jpg,https://oleks-netizen.github.io/product-images/11711001s/003.jpg,https://oleks-netizen.github.io/product-images/11711001s/004.jpg,https://oleks-netizen.github.io/product-images/11711001s/005.jpg,https://oleks-netizen.github.io/product-images/11711001s/006.jpg,https://oleks-netizen.github.io/product-images/11711001s/007.jpg,https://oleks-netizen.github.io/product-images/11711001s/008.jpg,https://oleks-netizen.github.io/product-images/11711001s/009.jpg,https://oleks-netizen.github.io/product-images/11711001s/010.jpg,https://oleks-netizen.github.io/product-images/11711001s/011.jpg,https://oleks-netizen.github.io/product-images/11711001s/012.jpg,https://oleks-netizen.github.io/product-images/11711001s/013.jpg,https://oleks-netizen.github.io/product-images/11711001s/014.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LC47541-1</t>
+          <t>11711065g</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47541-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/007.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/008.jpg,https://oleks-netizen.github.io/product-images/LC47541-1/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711065g/001.jpg,https://oleks-netizen.github.io/product-images/11711065g/002.jpg,https://oleks-netizen.github.io/product-images/11711065g/003.jpg,https://oleks-netizen.github.io/product-images/11711065g/004.jpg,https://oleks-netizen.github.io/product-images/11711065g/005.jpg,https://oleks-netizen.github.io/product-images/11711065g/007.jpg,https://oleks-netizen.github.io/product-images/11711065g/008.jpg,https://oleks-netizen.github.io/product-images/11711065g/009.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -481,27 +481,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LC47541-93</t>
+          <t>11711065s</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47541-93/001.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/002.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/004.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/005.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/006.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/007.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/008.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/009.jpg,https://oleks-netizen.github.io/product-images/LC47541-93/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711065s/001.jpg,https://oleks-netizen.github.io/product-images/11711065s/002.jpg,https://oleks-netizen.github.io/product-images/11711065s/003.jpg,https://oleks-netizen.github.io/product-images/11711065s/005.jpg,https://oleks-netizen.github.io/product-images/11711065s/006.jpg,https://oleks-netizen.github.io/product-images/11711065s/007.jpg,https://oleks-netizen.github.io/product-images/11711065s/008.jpg,https://oleks-netizen.github.io/product-images/11711065s/009.jpg,https://oleks-netizen.github.io/product-images/11711065s/010.jpg,https://oleks-netizen.github.io/product-images/11711065s/011.jpg,https://oleks-netizen.github.io/product-images/11711065s/012.jpg,https://oleks-netizen.github.io/product-images/11711065s/013.jpg,https://oleks-netizen.github.io/product-images/11711065s/014.jpg,https://oleks-netizen.github.io/product-images/11711065s/015.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LC47554-1</t>
+          <t>11711702g</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47554-1/001.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/002.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/003.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/004.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/005.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/006.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/007.jpg,https://oleks-netizen.github.io/product-images/LC47554-1/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711702g/001.jpg,https://oleks-netizen.github.io/product-images/11711702g/003.jpg,https://oleks-netizen.github.io/product-images/11711702g/004.jpg,https://oleks-netizen.github.io/product-images/11711702g/005.jpg,https://oleks-netizen.github.io/product-images/11711702g/006.jpg,https://oleks-netizen.github.io/product-images/11711702g/007.jpg,https://oleks-netizen.github.io/product-images/11711702g/008.jpg,https://oleks-netizen.github.io/product-images/11711702g/009.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -511,27 +511,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LC47632F-1C</t>
+          <t>11711707s</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47632F-1C/001.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/002.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/003.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/004.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/005.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/006.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/007.jpg,https://oleks-netizen.github.io/product-images/LC47632F-1C/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711707s/001.jpg,https://oleks-netizen.github.io/product-images/11711707s/002.jpg,https://oleks-netizen.github.io/product-images/11711707s/003.jpg,https://oleks-netizen.github.io/product-images/11711707s/005.jpg,https://oleks-netizen.github.io/product-images/11711707s/006.jpg,https://oleks-netizen.github.io/product-images/11711707s/007.jpg,https://oleks-netizen.github.io/product-images/11711707s/008.jpg,https://oleks-netizen.github.io/product-images/11711707s/009.jpg,https://oleks-netizen.github.io/product-images/11711707s/010.jpg,https://oleks-netizen.github.io/product-images/11711707s/011.jpg,https://oleks-netizen.github.io/product-images/11711707s/012.jpg,https://oleks-netizen.github.io/product-images/11711707s/013.jpg,https://oleks-netizen.github.io/product-images/11711707s/014.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LC47832-1C</t>
+          <t>11711710g</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47832-1C/001.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/002.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/003.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/004.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/005.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/006.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/007.jpg,https://oleks-netizen.github.io/product-images/LC47832-1C/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711710g/001.jpg,https://oleks-netizen.github.io/product-images/11711710g/003.jpg,https://oleks-netizen.github.io/product-images/11711710g/004.jpg,https://oleks-netizen.github.io/product-images/11711710g/005.jpg,https://oleks-netizen.github.io/product-images/11711710g/006.jpg,https://oleks-netizen.github.io/product-images/11711710g/007.jpg,https://oleks-netizen.github.io/product-images/11711710g/008.jpg,https://oleks-netizen.github.io/product-images/11711710g/009.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -541,46 +541,691 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LC47832-93</t>
+          <t>11711715g</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47832-93/001.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/002.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/003.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/004.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/005.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/006.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/007.jpg,https://oleks-netizen.github.io/product-images/LC47832-93/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711715g/001.jpg,https://oleks-netizen.github.io/product-images/11711715g/003.jpg,https://oleks-netizen.github.io/product-images/11711715g/004.jpg,https://oleks-netizen.github.io/product-images/11711715g/005.jpg,https://oleks-netizen.github.io/product-images/11711715g/006.jpg,https://oleks-netizen.github.io/product-images/11711715g/007.jpg,https://oleks-netizen.github.io/product-images/11711715g/008.jpg,https://oleks-netizen.github.io/product-images/11711715g/009.jpg,https://oleks-netizen.github.io/product-images/11711715g/010.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LC47891-1C</t>
+          <t>11711715s</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/LC47891-1C/001.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/002.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/003.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/004.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/005.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/006.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/007.jpg,https://oleks-netizen.github.io/product-images/LC47891-1C/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711715s/001.jpg,https://oleks-netizen.github.io/product-images/11711715s/002.jpg,https://oleks-netizen.github.io/product-images/11711715s/003.jpg,https://oleks-netizen.github.io/product-images/11711715s/005.jpg,https://oleks-netizen.github.io/product-images/11711715s/006.jpg,https://oleks-netizen.github.io/product-images/11711715s/007.jpg,https://oleks-netizen.github.io/product-images/11711715s/008.jpg,https://oleks-netizen.github.io/product-images/11711715s/009.jpg,https://oleks-netizen.github.io/product-images/11711715s/010.jpg,https://oleks-netizen.github.io/product-images/11711715s/011.jpg,https://oleks-netizen.github.io/product-images/11711715s/012.jpg,https://oleks-netizen.github.io/product-images/11711715s/013.jpg</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RJ-hold-3md</t>
+          <t>11711719g</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/RJ-hold-3md/001.jpg,https://oleks-netizen.github.io/product-images/RJ-hold-3md/002.jpg,https://oleks-netizen.github.io/product-images/RJ-hold-3md/003.jpg,https://oleks-netizen.github.io/product-images/RJ-hold-3md/005.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/11711719g/001.jpg,https://oleks-netizen.github.io/product-images/11711719g/002.jpg,https://oleks-netizen.github.io/product-images/11711719g/004.jpg,https://oleks-netizen.github.io/product-images/11711719g/005.jpg,https://oleks-netizen.github.io/product-images/11711719g/006.jpg,https://oleks-netizen.github.io/product-images/11711719g/007.jpg,https://oleks-netizen.github.io/product-images/11711719g/008.jpg,https://oleks-netizen.github.io/product-images/11711719g/009.jpg,https://oleks-netizen.github.io/product-images/11711719g/010.jpg,https://oleks-netizen.github.io/product-images/11711719g/011.jpg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11711719s</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/11711719s/001.jpg,https://oleks-netizen.github.io/product-images/11711719s/002.jpg,https://oleks-netizen.github.io/product-images/11711719s/003.jpg,https://oleks-netizen.github.io/product-images/11711719s/004.jpg,https://oleks-netizen.github.io/product-images/11711719s/006.jpg,https://oleks-netizen.github.io/product-images/11711719s/007.jpg,https://oleks-netizen.github.io/product-images/11711719s/008.jpg,https://oleks-netizen.github.io/product-images/11711719s/009.jpg,https://oleks-netizen.github.io/product-images/11711719s/010.jpg,https://oleks-netizen.github.io/product-images/11711719s/011.jpg,https://oleks-netizen.github.io/product-images/11711719s/012.jpg,https://oleks-netizen.github.io/product-images/11711719s/013.jpg,https://oleks-netizen.github.io/product-images/11711719s/014.jpg,https://oleks-netizen.github.io/product-images/11711719s/015.jpg</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11711720g</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/11711720g/001.jpg,https://oleks-netizen.github.io/product-images/11711720g/003.jpg,https://oleks-netizen.github.io/product-images/11711720g/004.jpg,https://oleks-netizen.github.io/product-images/11711720g/005.jpg,https://oleks-netizen.github.io/product-images/11711720g/006.jpg,https://oleks-netizen.github.io/product-images/11711720g/007.jpg,https://oleks-netizen.github.io/product-images/11711720g/008.jpg,https://oleks-netizen.github.io/product-images/11711720g/009.jpg,https://oleks-netizen.github.io/product-images/11711720g/010.jpg</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12123001g</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/12123001g/001.jpg,https://oleks-netizen.github.io/product-images/12123001g/002.jpg,https://oleks-netizen.github.io/product-images/12123001g/003.jpg,https://oleks-netizen.github.io/product-images/12123001g/004.jpg,https://oleks-netizen.github.io/product-images/12123001g/005.jpg,https://oleks-netizen.github.io/product-images/12123001g/006.jpg</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12123020g</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/12123020g/001.jpg,https://oleks-netizen.github.io/product-images/12123020g/003.jpg,https://oleks-netizen.github.io/product-images/12123020g/004.jpg,https://oleks-netizen.github.io/product-images/12123020g/005.jpg,https://oleks-netizen.github.io/product-images/12123020g/006.jpg,https://oleks-netizen.github.io/product-images/12123020g/007.jpg,https://oleks-netizen.github.io/product-images/12123020g/008.jpg,https://oleks-netizen.github.io/product-images/12123020g/009.jpg,https://oleks-netizen.github.io/product-images/12123020g/010.jpg</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>14511001s</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/14511001s/001.jpg,https://oleks-netizen.github.io/product-images/14511001s/002.jpg,https://oleks-netizen.github.io/product-images/14511001s/003.jpg,https://oleks-netizen.github.io/product-images/14511001s/005.jpg,https://oleks-netizen.github.io/product-images/14511001s/006.jpg,https://oleks-netizen.github.io/product-images/14511001s/007.jpg,https://oleks-netizen.github.io/product-images/14511001s/008.jpg,https://oleks-netizen.github.io/product-images/14511001s/009.jpg,https://oleks-netizen.github.io/product-images/14511001s/010.jpg</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>14511008s</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/14511008s/001.jpg,https://oleks-netizen.github.io/product-images/14511008s/002.jpg,https://oleks-netizen.github.io/product-images/14511008s/003.jpg,https://oleks-netizen.github.io/product-images/14511008s/004.jpg,https://oleks-netizen.github.io/product-images/14511008s/006.jpg,https://oleks-netizen.github.io/product-images/14511008s/007.jpg,https://oleks-netizen.github.io/product-images/14511008s/008.jpg,https://oleks-netizen.github.io/product-images/14511008s/009.jpg,https://oleks-netizen.github.io/product-images/14511008s/010.jpg,https://oleks-netizen.github.io/product-images/14511008s/011.jpg,https://oleks-netizen.github.io/product-images/14511008s/012.jpg</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>14511015</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/14511015/001.jpg,https://oleks-netizen.github.io/product-images/14511015/002.jpg,https://oleks-netizen.github.io/product-images/14511015/003.jpg,https://oleks-netizen.github.io/product-images/14511015/004.jpg,https://oleks-netizen.github.io/product-images/14511015/005.jpg,https://oleks-netizen.github.io/product-images/14511015/006.jpg,https://oleks-netizen.github.io/product-images/14511015/007.jpg,https://oleks-netizen.github.io/product-images/14511015/008.jpg,https://oleks-netizen.github.io/product-images/14511015/009.jpg,https://oleks-netizen.github.io/product-images/14511015/010.jpg,https://oleks-netizen.github.io/product-images/14511015/012.jpg,https://oleks-netizen.github.io/product-images/14511015/013.jpg,https://oleks-netizen.github.io/product-images/14511015/014.jpg</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14511020g</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/14511020g/001.jpg,https://oleks-netizen.github.io/product-images/14511020g/002.jpg,https://oleks-netizen.github.io/product-images/14511020g/004.jpg,https://oleks-netizen.github.io/product-images/14511020g/005.jpg,https://oleks-netizen.github.io/product-images/14511020g/006.jpg,https://oleks-netizen.github.io/product-images/14511020g/007.jpg,https://oleks-netizen.github.io/product-images/14511020g/008.jpg</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14511020s</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/14511020s/001.jpg,https://oleks-netizen.github.io/product-images/14511020s/003.jpg,https://oleks-netizen.github.io/product-images/14511020s/004.jpg,https://oleks-netizen.github.io/product-images/14511020s/005.jpg,https://oleks-netizen.github.io/product-images/14511020s/006.jpg,https://oleks-netizen.github.io/product-images/14511020s/007.jpg,https://oleks-netizen.github.io/product-images/14511020s/008.jpg,https://oleks-netizen.github.io/product-images/14511020s/009.jpg</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14511021g</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/14511021g/001.jpg,https://oleks-netizen.github.io/product-images/14511021g/003.jpg,https://oleks-netizen.github.io/product-images/14511021g/004.jpg,https://oleks-netizen.github.io/product-images/14511021g/005.jpg,https://oleks-netizen.github.io/product-images/14511021g/006.jpg,https://oleks-netizen.github.io/product-images/14511021g/007.jpg,https://oleks-netizen.github.io/product-images/14511021g/008.jpg,https://oleks-netizen.github.io/product-images/14511021g/009.jpg</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>15352020g</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/15352020g/001.jpg,https://oleks-netizen.github.io/product-images/15352020g/003.jpg,https://oleks-netizen.github.io/product-images/15352020g/004.jpg,https://oleks-netizen.github.io/product-images/15352020g/005.jpg,https://oleks-netizen.github.io/product-images/15352020g/006.jpg,https://oleks-netizen.github.io/product-images/15352020g/007.jpg,https://oleks-netizen.github.io/product-images/15352020g/008.jpg,https://oleks-netizen.github.io/product-images/15352020g/009.jpg,https://oleks-netizen.github.io/product-images/15352020g/010.jpg,https://oleks-netizen.github.io/product-images/15352020g/011.jpg,https://oleks-netizen.github.io/product-images/15352020g/012.jpg,https://oleks-netizen.github.io/product-images/15352020g/013.jpg,https://oleks-netizen.github.io/product-images/15352020g/014.jpg</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>15373001g</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/15373001g/001.jpg,https://oleks-netizen.github.io/product-images/15373001g/003.jpg,https://oleks-netizen.github.io/product-images/15373001g/004.jpg,https://oleks-netizen.github.io/product-images/15373001g/005.jpg,https://oleks-netizen.github.io/product-images/15373001g/006.jpg,https://oleks-netizen.github.io/product-images/15373001g/007.jpg,https://oleks-netizen.github.io/product-images/15373001g/008.jpg,https://oleks-netizen.github.io/product-images/15373001g/009.jpg,https://oleks-netizen.github.io/product-images/15373001g/010.jpg</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15373008</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/15373008/001.jpg,https://oleks-netizen.github.io/product-images/15373008/002.jpg,https://oleks-netizen.github.io/product-images/15373008/003.jpg,https://oleks-netizen.github.io/product-images/15373008/004.jpg,https://oleks-netizen.github.io/product-images/15373008/005.jpg,https://oleks-netizen.github.io/product-images/15373008/006.jpg,https://oleks-netizen.github.io/product-images/15373008/007.jpg,https://oleks-netizen.github.io/product-images/15373008/008.jpg,https://oleks-netizen.github.io/product-images/15373008/009.jpg,https://oleks-netizen.github.io/product-images/15373008/010.jpg,https://oleks-netizen.github.io/product-images/15373008/012.jpg,https://oleks-netizen.github.io/product-images/15373008/013.jpg,https://oleks-netizen.github.io/product-images/15373008/014.jpg,https://oleks-netizen.github.io/product-images/15373008/015.jpg,https://oleks-netizen.github.io/product-images/15373008/016.jpg</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>15373008g</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/15373008g/001.jpg,https://oleks-netizen.github.io/product-images/15373008g/003.jpg,https://oleks-netizen.github.io/product-images/15373008g/004.jpg,https://oleks-netizen.github.io/product-images/15373008g/005.jpg,https://oleks-netizen.github.io/product-images/15373008g/006.jpg,https://oleks-netizen.github.io/product-images/15373008g/007.jpg,https://oleks-netizen.github.io/product-images/15373008g/008.jpg,https://oleks-netizen.github.io/product-images/15373008g/009.jpg,https://oleks-netizen.github.io/product-images/15373008g/010.jpg</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15373020g</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/15373020g/001.jpg,https://oleks-netizen.github.io/product-images/15373020g/002.jpg,https://oleks-netizen.github.io/product-images/15373020g/003.jpg,https://oleks-netizen.github.io/product-images/15373020g/004.jpg,https://oleks-netizen.github.io/product-images/15373020g/005.jpg,https://oleks-netizen.github.io/product-images/15373020g/006.jpg,https://oleks-netizen.github.io/product-images/15373020g/007.jpg,https://oleks-netizen.github.io/product-images/15373020g/008.jpg</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2220-05-31</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/2220-05-31/001.jpg,https://oleks-netizen.github.io/product-images/2220-05-31/002.jpg,https://oleks-netizen.github.io/product-images/2220-05-31/003.jpg,https://oleks-netizen.github.io/product-images/2220-05-31/004.jpg,https://oleks-netizen.github.io/product-images/2220-05-31/005.jpg</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>25000001g</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000001g/001.jpg,https://oleks-netizen.github.io/product-images/25000001g/002.jpg,https://oleks-netizen.github.io/product-images/25000001g/003.jpg,https://oleks-netizen.github.io/product-images/25000001g/004.jpg,https://oleks-netizen.github.io/product-images/25000001g/005.jpg,https://oleks-netizen.github.io/product-images/25000001g/006.jpg,https://oleks-netizen.github.io/product-images/25000001g/007.jpg,https://oleks-netizen.github.io/product-images/25000001g/008.jpg</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>25000001s</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000001s/001.jpg,https://oleks-netizen.github.io/product-images/25000001s/003.jpg,https://oleks-netizen.github.io/product-images/25000001s/004.jpg,https://oleks-netizen.github.io/product-images/25000001s/005.jpg,https://oleks-netizen.github.io/product-images/25000001s/006.jpg,https://oleks-netizen.github.io/product-images/25000001s/007.jpg,https://oleks-netizen.github.io/product-images/25000001s/008.jpg,https://oleks-netizen.github.io/product-images/25000001s/009.jpg,https://oleks-netizen.github.io/product-images/25000001s/010.jpg,https://oleks-netizen.github.io/product-images/25000001s/011.jpg,https://oleks-netizen.github.io/product-images/25000001s/012.jpg,https://oleks-netizen.github.io/product-images/25000001s/013.jpg,https://oleks-netizen.github.io/product-images/25000001s/014.jpg</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>25000010s</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000010s/001.jpg,https://oleks-netizen.github.io/product-images/25000010s/002.jpg,https://oleks-netizen.github.io/product-images/25000010s/003.jpg,https://oleks-netizen.github.io/product-images/25000010s/005.jpg,https://oleks-netizen.github.io/product-images/25000010s/006.jpg,https://oleks-netizen.github.io/product-images/25000010s/007.jpg,https://oleks-netizen.github.io/product-images/25000010s/008.jpg,https://oleks-netizen.github.io/product-images/25000010s/009.jpg,https://oleks-netizen.github.io/product-images/25000010s/010.jpg,https://oleks-netizen.github.io/product-images/25000010s/011.jpg,https://oleks-netizen.github.io/product-images/25000010s/012.jpg,https://oleks-netizen.github.io/product-images/25000010s/013.jpg,https://oleks-netizen.github.io/product-images/25000010s/014.jpg,https://oleks-netizen.github.io/product-images/25000010s/015.jpg</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>25000030s</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000030s/001.jpg,https://oleks-netizen.github.io/product-images/25000030s/003.jpg,https://oleks-netizen.github.io/product-images/25000030s/004.jpg,https://oleks-netizen.github.io/product-images/25000030s/005.jpg,https://oleks-netizen.github.io/product-images/25000030s/006.jpg,https://oleks-netizen.github.io/product-images/25000030s/007.jpg,https://oleks-netizen.github.io/product-images/25000030s/008.jpg,https://oleks-netizen.github.io/product-images/25000030s/009.jpg,https://oleks-netizen.github.io/product-images/25000030s/010.jpg,https://oleks-netizen.github.io/product-images/25000030s/011.jpg,https://oleks-netizen.github.io/product-images/25000030s/012.jpg</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>25000064g</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000064g/001.jpg,https://oleks-netizen.github.io/product-images/25000064g/003.jpg,https://oleks-netizen.github.io/product-images/25000064g/004.jpg,https://oleks-netizen.github.io/product-images/25000064g/005.jpg,https://oleks-netizen.github.io/product-images/25000064g/006.jpg,https://oleks-netizen.github.io/product-images/25000064g/007.jpg,https://oleks-netizen.github.io/product-images/25000064g/008.jpg,https://oleks-netizen.github.io/product-images/25000064g/009.jpg,https://oleks-netizen.github.io/product-images/25000064g/010.jpg,https://oleks-netizen.github.io/product-images/25000064g/011.jpg,https://oleks-netizen.github.io/product-images/25000064g/012.jpg,https://oleks-netizen.github.io/product-images/25000064g/013.jpg</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>25000064s</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000064s/001.jpg,https://oleks-netizen.github.io/product-images/25000064s/003.jpg,https://oleks-netizen.github.io/product-images/25000064s/004.jpg,https://oleks-netizen.github.io/product-images/25000064s/005.jpg,https://oleks-netizen.github.io/product-images/25000064s/006.jpg,https://oleks-netizen.github.io/product-images/25000064s/007.jpg,https://oleks-netizen.github.io/product-images/25000064s/008.jpg,https://oleks-netizen.github.io/product-images/25000064s/009.jpg,https://oleks-netizen.github.io/product-images/25000064s/010.jpg,https://oleks-netizen.github.io/product-images/25000064s/011.jpg,https://oleks-netizen.github.io/product-images/25000064s/012.jpg,https://oleks-netizen.github.io/product-images/25000064s/013.jpg,https://oleks-netizen.github.io/product-images/25000064s/014.jpg,https://oleks-netizen.github.io/product-images/25000064s/015.jpg</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>25000264g</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000264g/001.jpg,https://oleks-netizen.github.io/product-images/25000264g/002.jpg,https://oleks-netizen.github.io/product-images/25000264g/003.jpg,https://oleks-netizen.github.io/product-images/25000264g/004.jpg,https://oleks-netizen.github.io/product-images/25000264g/005.jpg,https://oleks-netizen.github.io/product-images/25000264g/006.jpg,https://oleks-netizen.github.io/product-images/25000264g/007.jpg,https://oleks-netizen.github.io/product-images/25000264g/008.jpg,https://oleks-netizen.github.io/product-images/25000264g/009.jpg,https://oleks-netizen.github.io/product-images/25000264g/010.jpg</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>25000264s</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000264s/001.jpg,https://oleks-netizen.github.io/product-images/25000264s/002.jpg,https://oleks-netizen.github.io/product-images/25000264s/003.jpg,https://oleks-netizen.github.io/product-images/25000264s/005.jpg,https://oleks-netizen.github.io/product-images/25000264s/006.jpg,https://oleks-netizen.github.io/product-images/25000264s/007.jpg,https://oleks-netizen.github.io/product-images/25000264s/008.jpg,https://oleks-netizen.github.io/product-images/25000264s/009.jpg,https://oleks-netizen.github.io/product-images/25000264s/010.jpg,https://oleks-netizen.github.io/product-images/25000264s/011.jpg,https://oleks-netizen.github.io/product-images/25000264s/012.jpg,https://oleks-netizen.github.io/product-images/25000264s/013.jpg,https://oleks-netizen.github.io/product-images/25000264s/014.jpg</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>25000506g</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000506g/001.jpg,https://oleks-netizen.github.io/product-images/25000506g/002.jpg,https://oleks-netizen.github.io/product-images/25000506g/003.jpg,https://oleks-netizen.github.io/product-images/25000506g/004.jpg,https://oleks-netizen.github.io/product-images/25000506g/005.jpg,https://oleks-netizen.github.io/product-images/25000506g/006.jpg,https://oleks-netizen.github.io/product-images/25000506g/007.jpg,https://oleks-netizen.github.io/product-images/25000506g/008.jpg,https://oleks-netizen.github.io/product-images/25000506g/009.jpg,https://oleks-netizen.github.io/product-images/25000506g/010.jpg</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>25000514g</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000514g/001.jpg,https://oleks-netizen.github.io/product-images/25000514g/003.jpg,https://oleks-netizen.github.io/product-images/25000514g/004.jpg,https://oleks-netizen.github.io/product-images/25000514g/005.jpg,https://oleks-netizen.github.io/product-images/25000514g/006.jpg,https://oleks-netizen.github.io/product-images/25000514g/007.jpg,https://oleks-netizen.github.io/product-images/25000514g/008.jpg,https://oleks-netizen.github.io/product-images/25000514g/009.jpg,https://oleks-netizen.github.io/product-images/25000514g/010.jpg,https://oleks-netizen.github.io/product-images/25000514g/011.jpg,https://oleks-netizen.github.io/product-images/25000514g/012.jpg,https://oleks-netizen.github.io/product-images/25000514g/013.jpg,https://oleks-netizen.github.io/product-images/25000514g/014.jpg</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>25000515s</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25000515s/001.jpg,https://oleks-netizen.github.io/product-images/25000515s/002.jpg,https://oleks-netizen.github.io/product-images/25000515s/003.jpg,https://oleks-netizen.github.io/product-images/25000515s/005.jpg,https://oleks-netizen.github.io/product-images/25000515s/006.jpg,https://oleks-netizen.github.io/product-images/25000515s/007.jpg,https://oleks-netizen.github.io/product-images/25000515s/008.jpg,https://oleks-netizen.github.io/product-images/25000515s/009.jpg,https://oleks-netizen.github.io/product-images/25000515s/010.jpg,https://oleks-netizen.github.io/product-images/25000515s/011.jpg,https://oleks-netizen.github.io/product-images/25000515s/012.jpg,https://oleks-netizen.github.io/product-images/25000515s/013.jpg,https://oleks-netizen.github.io/product-images/25000515s/014.jpg,https://oleks-netizen.github.io/product-images/25000515s/015.jpg,https://oleks-netizen.github.io/product-images/25000515s/016.jpg</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>25018001g</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25018001g/001.jpg,https://oleks-netizen.github.io/product-images/25018001g/003.jpg,https://oleks-netizen.github.io/product-images/25018001g/004.jpg,https://oleks-netizen.github.io/product-images/25018001g/005.jpg,https://oleks-netizen.github.io/product-images/25018001g/006.jpg,https://oleks-netizen.github.io/product-images/25018001g/007.jpg,https://oleks-netizen.github.io/product-images/25018001g/008.jpg,https://oleks-netizen.github.io/product-images/25018001g/009.jpg</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>25058001g</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25058001g/001.jpg,https://oleks-netizen.github.io/product-images/25058001g/002.jpg,https://oleks-netizen.github.io/product-images/25058001g/003.jpg,https://oleks-netizen.github.io/product-images/25058001g/004.jpg,https://oleks-netizen.github.io/product-images/25058001g/005.jpg,https://oleks-netizen.github.io/product-images/25058001g/006.jpg</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>25088001s</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25088001s/001.jpg,https://oleks-netizen.github.io/product-images/25088001s/002.jpg,https://oleks-netizen.github.io/product-images/25088001s/003.jpg,https://oleks-netizen.github.io/product-images/25088001s/004.jpg,https://oleks-netizen.github.io/product-images/25088001s/005.jpg,https://oleks-netizen.github.io/product-images/25088001s/006.jpg,https://oleks-netizen.github.io/product-images/25088001s/007.jpg,https://oleks-netizen.github.io/product-images/25088001s/008.jpg,https://oleks-netizen.github.io/product-images/25088001s/009.jpg,https://oleks-netizen.github.io/product-images/25088001s/010.jpg</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>25428001g</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/25428001g/001.jpg,https://oleks-netizen.github.io/product-images/25428001g/002.jpg,https://oleks-netizen.github.io/product-images/25428001g/004.jpg,https://oleks-netizen.github.io/product-images/25428001g/005.jpg,https://oleks-netizen.github.io/product-images/25428001g/006.jpg,https://oleks-netizen.github.io/product-images/25428001g/007.jpg,https://oleks-netizen.github.io/product-images/25428001g/008.jpg,https://oleks-netizen.github.io/product-images/25428001g/009.jpg,https://oleks-netizen.github.io/product-images/25428001g/010.jpg,https://oleks-netizen.github.io/product-images/25428001g/011.jpg</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>35312001g</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/35312001g/001.jpg,https://oleks-netizen.github.io/product-images/35312001g/002.jpg,https://oleks-netizen.github.io/product-images/35312001g/004.jpg,https://oleks-netizen.github.io/product-images/35312001g/005.jpg,https://oleks-netizen.github.io/product-images/35312001g/006.jpg,https://oleks-netizen.github.io/product-images/35312001g/007.jpg,https://oleks-netizen.github.io/product-images/35312001g/008.jpg,https://oleks-netizen.github.io/product-images/35312001g/009.jpg</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>35312008g</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/35312008g/001.jpg,https://oleks-netizen.github.io/product-images/35312008g/002.jpg,https://oleks-netizen.github.io/product-images/35312008g/003.jpg,https://oleks-netizen.github.io/product-images/35312008g/004.jpg,https://oleks-netizen.github.io/product-images/35312008g/005.jpg,https://oleks-netizen.github.io/product-images/35312008g/006.jpg,https://oleks-netizen.github.io/product-images/35312008g/007.jpg,https://oleks-netizen.github.io/product-images/35312008g/008.jpg</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>L20688-1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20688-1/001.jpg,https://oleks-netizen.github.io/product-images/L20688-1/002.jpg,https://oleks-netizen.github.io/product-images/L20688-1/004.jpg,https://oleks-netizen.github.io/product-images/L20688-1/005.jpg,https://oleks-netizen.github.io/product-images/L20688-1/006.jpg,https://oleks-netizen.github.io/product-images/L20688-1/007.jpg,https://oleks-netizen.github.io/product-images/L20688-1/008.jpg,https://oleks-netizen.github.io/product-images/L20688-1/009.jpg,https://oleks-netizen.github.io/product-images/L20688-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>L20688-15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20688-15/001.jpg,https://oleks-netizen.github.io/product-images/L20688-15/002.jpg,https://oleks-netizen.github.io/product-images/L20688-15/004.jpg,https://oleks-netizen.github.io/product-images/L20688-15/005.jpg,https://oleks-netizen.github.io/product-images/L20688-15/006.jpg,https://oleks-netizen.github.io/product-images/L20688-15/007.jpg,https://oleks-netizen.github.io/product-images/L20688-15/008.jpg,https://oleks-netizen.github.io/product-images/L20688-15/009.jpg,https://oleks-netizen.github.io/product-images/L20688-15/010.jpg</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>L20688-2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20688-2/001.jpg,https://oleks-netizen.github.io/product-images/L20688-2/002.jpg,https://oleks-netizen.github.io/product-images/L20688-2/004.jpg,https://oleks-netizen.github.io/product-images/L20688-2/005.jpg,https://oleks-netizen.github.io/product-images/L20688-2/006.jpg,https://oleks-netizen.github.io/product-images/L20688-2/007.jpg,https://oleks-netizen.github.io/product-images/L20688-2/008.jpg,https://oleks-netizen.github.io/product-images/L20688-2/009.jpg,https://oleks-netizen.github.io/product-images/L20688-2/010.jpg</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>L20702-1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20702-1/001.jpg,https://oleks-netizen.github.io/product-images/L20702-1/002.jpg,https://oleks-netizen.github.io/product-images/L20702-1/004.jpg,https://oleks-netizen.github.io/product-images/L20702-1/005.jpg,https://oleks-netizen.github.io/product-images/L20702-1/006.jpg,https://oleks-netizen.github.io/product-images/L20702-1/007.jpg,https://oleks-netizen.github.io/product-images/L20702-1/008.jpg,https://oleks-netizen.github.io/product-images/L20702-1/009.jpg,https://oleks-netizen.github.io/product-images/L20702-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>L20702-46</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20702-46/001.jpg,https://oleks-netizen.github.io/product-images/L20702-46/002.jpg,https://oleks-netizen.github.io/product-images/L20702-46/004.jpg,https://oleks-netizen.github.io/product-images/L20702-46/005.jpg,https://oleks-netizen.github.io/product-images/L20702-46/006.jpg,https://oleks-netizen.github.io/product-images/L20702-46/007.jpg,https://oleks-netizen.github.io/product-images/L20702-46/008.jpg,https://oleks-netizen.github.io/product-images/L20702-46/009.jpg,https://oleks-netizen.github.io/product-images/L20702-46/010.jpg</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>L20731-1</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/L20731-1/001.jpg,https://oleks-netizen.github.io/product-images/L20731-1/002.jpg,https://oleks-netizen.github.io/product-images/L20731-1/004.jpg,https://oleks-netizen.github.io/product-images/L20731-1/005.jpg,https://oleks-netizen.github.io/product-images/L20731-1/006.jpg,https://oleks-netizen.github.io/product-images/L20731-1/007.jpg,https://oleks-netizen.github.io/product-images/L20731-1/008.jpg</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LC46063-1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/LC46063-1/001.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/002.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/004.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/005.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/006.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/007.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/008.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/009.jpg,https://oleks-netizen.github.io/product-images/LC46063-1/010.jpg</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>RB-7281-3md</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RB-7281-3md/001.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/002.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/003.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/004.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/005.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/006.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/007.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/008.jpg,https://oleks-netizen.github.io/product-images/RB-7281-3md/009.jpg</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>RE-1240-4lx</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/RE-1240-4lx/001.jpg,https://oleks-netizen.github.io/product-images/RE-1240-4lx/002.jpg,https://oleks-netizen.github.io/product-images/RE-1240-4lx/003.jpg,https://oleks-netizen.github.io/product-images/RE-1240-4lx/005.jpg,https://oleks-netizen.github.io/product-images/RE-1240-4lx/006.jpg</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TW-Kim-caramel</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/TW-Kim-caramel/001.jpg</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update 2026-09-02 09:40:30
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,240 +436,120 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>64807 BLK</t>
+          <t>53405008</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/64807 BLK/001.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/002.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/003.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/004.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/005.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/006.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/008.jpg,https://oleks-netizen.github.io/product-images/64807 BLK/009.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53405008/001.jpg,https://oleks-netizen.github.io/product-images/53405008/002.jpg,https://oleks-netizen.github.io/product-images/53405008/003.jpg,https://oleks-netizen.github.io/product-images/53405008/005.jpg,https://oleks-netizen.github.io/product-images/53405008/006.jpg,https://oleks-netizen.github.io/product-images/53405008/007.jpg,https://oleks-netizen.github.io/product-images/53405008/008.jpg,https://oleks-netizen.github.io/product-images/53405008/009.jpg,https://oleks-netizen.github.io/product-images/53405008/010.jpg,https://oleks-netizen.github.io/product-images/53405008/011.jpg,https://oleks-netizen.github.io/product-images/53405008/012.jpg,https://oleks-netizen.github.io/product-images/53405008/013.jpg,https://oleks-netizen.github.io/product-images/53405008/014.jpg,https://oleks-netizen.github.io/product-images/53405008/015.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>720 BLK</t>
+          <t>53405020</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/720 BLK/001.jpg,https://oleks-netizen.github.io/product-images/720 BLK/002.jpg,https://oleks-netizen.github.io/product-images/720 BLK/003.jpg,https://oleks-netizen.github.io/product-images/720 BLK/004.jpg,https://oleks-netizen.github.io/product-images/720 BLK/005.jpg,https://oleks-netizen.github.io/product-images/720 BLK/006.jpg,https://oleks-netizen.github.io/product-images/720 BLK/007.jpg,https://oleks-netizen.github.io/product-images/720 BLK/008.jpg,https://oleks-netizen.github.io/product-images/720 BLK/009.jpg,https://oleks-netizen.github.io/product-images/720 BLK/010.jpg,https://oleks-netizen.github.io/product-images/720 BLK/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53405020/001.jpg,https://oleks-netizen.github.io/product-images/53405020/003.jpg,https://oleks-netizen.github.io/product-images/53405020/004.jpg,https://oleks-netizen.github.io/product-images/53405020/005.jpg,https://oleks-netizen.github.io/product-images/53405020/006.jpg,https://oleks-netizen.github.io/product-images/53405020/007.jpg,https://oleks-netizen.github.io/product-images/53405020/008.jpg,https://oleks-netizen.github.io/product-images/53405020/009.jpg,https://oleks-netizen.github.io/product-images/53405020/010.jpg,https://oleks-netizen.github.io/product-images/53405020/011.jpg,https://oleks-netizen.github.io/product-images/53405020/012.jpg,https://oleks-netizen.github.io/product-images/53405020/013.jpg,https://oleks-netizen.github.io/product-images/53405020/014.jpg,https://oleks-netizen.github.io/product-images/53405020/015.jpg,https://oleks-netizen.github.io/product-images/53405020/016.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>720 BR</t>
+          <t>53405064</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/720 BR/001.jpg,https://oleks-netizen.github.io/product-images/720 BR/002.jpg,https://oleks-netizen.github.io/product-images/720 BR/003.jpg,https://oleks-netizen.github.io/product-images/720 BR/004.jpg,https://oleks-netizen.github.io/product-images/720 BR/005.jpg,https://oleks-netizen.github.io/product-images/720 BR/006.jpg,https://oleks-netizen.github.io/product-images/720 BR/007.jpg,https://oleks-netizen.github.io/product-images/720 BR/009.jpg,https://oleks-netizen.github.io/product-images/720 BR/010.jpg,https://oleks-netizen.github.io/product-images/720 BR/011.jpg,https://oleks-netizen.github.io/product-images/720 BR/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53405064/001.jpg,https://oleks-netizen.github.io/product-images/53405064/002.jpg,https://oleks-netizen.github.io/product-images/53405064/003.jpg,https://oleks-netizen.github.io/product-images/53405064/004.jpg,https://oleks-netizen.github.io/product-images/53405064/005.jpg,https://oleks-netizen.github.io/product-images/53405064/006.jpg,https://oleks-netizen.github.io/product-images/53405064/007.jpg,https://oleks-netizen.github.io/product-images/53405064/008.jpg,https://oleks-netizen.github.io/product-images/53405064/009.jpg,https://oleks-netizen.github.io/product-images/53405064/011.jpg,https://oleks-netizen.github.io/product-images/53405064/012.jpg,https://oleks-netizen.github.io/product-images/53405064/013.jpg,https://oleks-netizen.github.io/product-images/53405064/014.jpg,https://oleks-netizen.github.io/product-images/53405064/015.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>720 OIL BR</t>
+          <t>53405510</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/720 OIL BR/001.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/002.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/003.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/004.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/005.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/006.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/007.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/009.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/010.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/011.jpg,https://oleks-netizen.github.io/product-images/720 OIL BR/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53405510/001.jpg,https://oleks-netizen.github.io/product-images/53405510/002.jpg,https://oleks-netizen.github.io/product-images/53405510/004.jpg,https://oleks-netizen.github.io/product-images/53405510/005.jpg,https://oleks-netizen.github.io/product-images/53405510/006.jpg,https://oleks-netizen.github.io/product-images/53405510/007.jpg,https://oleks-netizen.github.io/product-images/53405510/008.jpg,https://oleks-netizen.github.io/product-images/53405510/009.jpg,https://oleks-netizen.github.io/product-images/53405510/010.jpg,https://oleks-netizen.github.io/product-images/53405510/011.jpg,https://oleks-netizen.github.io/product-images/53405510/012.jpg,https://oleks-netizen.github.io/product-images/53405510/013.jpg,https://oleks-netizen.github.io/product-images/53405510/014.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>720 OIL TAN</t>
+          <t>53405515</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/720 OIL TAN/001.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/002.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/003.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/004.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/005.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/006.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/007.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/008.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/009.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/011.jpg,https://oleks-netizen.github.io/product-images/720 OIL TAN/012.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/53405515/001.jpg,https://oleks-netizen.github.io/product-images/53405515/002.jpg,https://oleks-netizen.github.io/product-images/53405515/003.jpg,https://oleks-netizen.github.io/product-images/53405515/004.jpg,https://oleks-netizen.github.io/product-images/53405515/005.jpg,https://oleks-netizen.github.io/product-images/53405515/006.jpg,https://oleks-netizen.github.io/product-images/53405515/008.jpg,https://oleks-netizen.github.io/product-images/53405515/009.jpg,https://oleks-netizen.github.io/product-images/53405515/010.jpg,https://oleks-netizen.github.io/product-images/53405515/011.jpg,https://oleks-netizen.github.io/product-images/53405515/012.jpg,https://oleks-netizen.github.io/product-images/53405515/013.jpg,https://oleks-netizen.github.io/product-images/53405515/014.jpg,https://oleks-netizen.github.io/product-images/53405515/015.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>721 BLK</t>
+          <t>90321510</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/721 BLK/001.jpg,https://oleks-netizen.github.io/product-images/721 BLK/002.jpg,https://oleks-netizen.github.io/product-images/721 BLK/003.jpg,https://oleks-netizen.github.io/product-images/721 BLK/004.jpg,https://oleks-netizen.github.io/product-images/721 BLK/005.jpg,https://oleks-netizen.github.io/product-images/721 BLK/006.jpg,https://oleks-netizen.github.io/product-images/721 BLK/007.jpg,https://oleks-netizen.github.io/product-images/721 BLK/008.jpg,https://oleks-netizen.github.io/product-images/721 BLK/009.jpg,https://oleks-netizen.github.io/product-images/721 BLK/010.jpg,https://oleks-netizen.github.io/product-images/721 BLK/011.jpg,https://oleks-netizen.github.io/product-images/721 BLK/013.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90321510/001.jpg,https://oleks-netizen.github.io/product-images/90321510/002.jpg,https://oleks-netizen.github.io/product-images/90321510/004.jpg,https://oleks-netizen.github.io/product-images/90321510/005.jpg,https://oleks-netizen.github.io/product-images/90321510/006.jpg,https://oleks-netizen.github.io/product-images/90321510/007.jpg,https://oleks-netizen.github.io/product-images/90321510/008.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8150 BROWN</t>
+          <t>90321515</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/8150 BROWN/001.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/002.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/003.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/004.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/005.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/006.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/007.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/008.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/009.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/010.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/011.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/012.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/013.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/015.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/016.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/017.jpg,https://oleks-netizen.github.io/product-images/8150 BROWN/018.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90321515/001.jpg,https://oleks-netizen.github.io/product-images/90321515/002.jpg,https://oleks-netizen.github.io/product-images/90321515/003.jpg,https://oleks-netizen.github.io/product-images/90321515/004.jpg,https://oleks-netizen.github.io/product-images/90321515/005.jpg,https://oleks-netizen.github.io/product-images/90321515/006.jpg,https://oleks-netizen.github.io/product-images/90321515/007.jpg,https://oleks-netizen.github.io/product-images/90321515/008.jpg,https://oleks-netizen.github.io/product-images/90321515/010.jpg,https://oleks-netizen.github.io/product-images/90321515/011.jpg,https://oleks-netizen.github.io/product-images/90321515/012.jpg,https://oleks-netizen.github.io/product-images/90321515/013.jpg,https://oleks-netizen.github.io/product-images/90321515/014.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G34 HONEY</t>
+          <t>90321714</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/G34 HONEY/001.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/002.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/003.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/004.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/005.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/006.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/007.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/008.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/009.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/010.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/011.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/012.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/014.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/015.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/016.jpg,https://oleks-netizen.github.io/product-images/G34 HONEY/017.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/90321714/001.jpg,https://oleks-netizen.github.io/product-images/90321714/002.jpg,https://oleks-netizen.github.io/product-images/90321714/004.jpg,https://oleks-netizen.github.io/product-images/90321714/005.jpg,https://oleks-netizen.github.io/product-images/90321714/006.jpg,https://oleks-netizen.github.io/product-images/90321714/007.jpg,https://oleks-netizen.github.io/product-images/90321714/008.jpg,https://oleks-netizen.github.io/product-images/90321714/009.jpg,https://oleks-netizen.github.io/product-images/90321714/010.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>K45 BLK</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/K45 BLK/001.jpg,https://oleks-netizen.github.io/product-images/K45 BLK/002.jpg,https://oleks-netizen.github.io/product-images/K45 BLK/003.jpg,https://oleks-netizen.github.io/product-images/K45 BLK/004.jpg,https://oleks-netizen.github.io/product-images/K45 BLK/006.jpg</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>K45 BRN</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/K45 BRN/001.jpg,https://oleks-netizen.github.io/product-images/K45 BRN/002.jpg,https://oleks-netizen.github.io/product-images/K45 BRN/003.jpg,https://oleks-netizen.github.io/product-images/K45 BRN/004.jpg,https://oleks-netizen.github.io/product-images/K45 BRN/006.jpg</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>P68 BLK</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/P68 BLK/001.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/002.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/003.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/004.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/005.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/006.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/007.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/008.jpg,https://oleks-netizen.github.io/product-images/P68 BLK/010.jpg</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>P68 GREEN</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/P68 GREEN/001.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/002.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/003.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/004.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/005.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/006.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/007.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/008.jpg,https://oleks-netizen.github.io/product-images/P68 GREEN/010.jpg</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TC92 BLK</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/TC92 BLK/001.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/002.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/003.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/004.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/005.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/006.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/007.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/009.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/010.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/011.jpg,https://oleks-netizen.github.io/product-images/TC92 BLK/012.jpg</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TC92 H_TAN</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/TC92 H_TAN/001.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/002.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/003.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/004.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/005.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/006.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/007.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/009.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/010.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/011.jpg,https://oleks-netizen.github.io/product-images/TC92 H_TAN/012.jpg</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TC93 CHT_BRN</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/001.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/002.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/003.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/004.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/005.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/006.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/007.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/008.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/009.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/010.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/011.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/013.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/014.jpg,https://oleks-netizen.github.io/product-images/TC93 CHT_BRN/015.jpg</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>X37 BLK</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://oleks-netizen.github.io/product-images/X37 BLK/001.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/002.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/003.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/004.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/005.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/007.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/008.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/009.jpg,https://oleks-netizen.github.io/product-images/X37 BLK/010.jpg</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto update 2026-10-25 18:42:33
</commit_message>
<xml_diff>
--- a/articles_summary.xlsx
+++ b/articles_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,121 +436,361 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>53405008</t>
+          <t>BN-GC-19-g-kr</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53405008/001.jpg,https://oleks-netizen.github.io/product-images/53405008/002.jpg,https://oleks-netizen.github.io/product-images/53405008/003.jpg,https://oleks-netizen.github.io/product-images/53405008/005.jpg,https://oleks-netizen.github.io/product-images/53405008/006.jpg,https://oleks-netizen.github.io/product-images/53405008/007.jpg,https://oleks-netizen.github.io/product-images/53405008/008.jpg,https://oleks-netizen.github.io/product-images/53405008/009.jpg,https://oleks-netizen.github.io/product-images/53405008/010.jpg,https://oleks-netizen.github.io/product-images/53405008/011.jpg,https://oleks-netizen.github.io/product-images/53405008/012.jpg,https://oleks-netizen.github.io/product-images/53405008/013.jpg,https://oleks-netizen.github.io/product-images/53405008/014.jpg,https://oleks-netizen.github.io/product-images/53405008/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-g-kr/004.jpg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>53405020</t>
+          <t>BN-GC-19-iz</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53405020/001.jpg,https://oleks-netizen.github.io/product-images/53405020/003.jpg,https://oleks-netizen.github.io/product-images/53405020/004.jpg,https://oleks-netizen.github.io/product-images/53405020/005.jpg,https://oleks-netizen.github.io/product-images/53405020/006.jpg,https://oleks-netizen.github.io/product-images/53405020/007.jpg,https://oleks-netizen.github.io/product-images/53405020/008.jpg,https://oleks-netizen.github.io/product-images/53405020/009.jpg,https://oleks-netizen.github.io/product-images/53405020/010.jpg,https://oleks-netizen.github.io/product-images/53405020/011.jpg,https://oleks-netizen.github.io/product-images/53405020/012.jpg,https://oleks-netizen.github.io/product-images/53405020/013.jpg,https://oleks-netizen.github.io/product-images/53405020/014.jpg,https://oleks-netizen.github.io/product-images/53405020/015.jpg,https://oleks-netizen.github.io/product-images/53405020/016.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-iz/004.jpg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>53405064</t>
+          <t>BN-GC-19-k-kr</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53405064/001.jpg,https://oleks-netizen.github.io/product-images/53405064/002.jpg,https://oleks-netizen.github.io/product-images/53405064/003.jpg,https://oleks-netizen.github.io/product-images/53405064/004.jpg,https://oleks-netizen.github.io/product-images/53405064/005.jpg,https://oleks-netizen.github.io/product-images/53405064/006.jpg,https://oleks-netizen.github.io/product-images/53405064/007.jpg,https://oleks-netizen.github.io/product-images/53405064/008.jpg,https://oleks-netizen.github.io/product-images/53405064/009.jpg,https://oleks-netizen.github.io/product-images/53405064/011.jpg,https://oleks-netizen.github.io/product-images/53405064/012.jpg,https://oleks-netizen.github.io/product-images/53405064/013.jpg,https://oleks-netizen.github.io/product-images/53405064/014.jpg,https://oleks-netizen.github.io/product-images/53405064/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-k-kr/004.jpg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>53405510</t>
+          <t>BN-GC-19-o</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53405510/001.jpg,https://oleks-netizen.github.io/product-images/53405510/002.jpg,https://oleks-netizen.github.io/product-images/53405510/004.jpg,https://oleks-netizen.github.io/product-images/53405510/005.jpg,https://oleks-netizen.github.io/product-images/53405510/006.jpg,https://oleks-netizen.github.io/product-images/53405510/007.jpg,https://oleks-netizen.github.io/product-images/53405510/008.jpg,https://oleks-netizen.github.io/product-images/53405510/009.jpg,https://oleks-netizen.github.io/product-images/53405510/010.jpg,https://oleks-netizen.github.io/product-images/53405510/011.jpg,https://oleks-netizen.github.io/product-images/53405510/012.jpg,https://oleks-netizen.github.io/product-images/53405510/013.jpg,https://oleks-netizen.github.io/product-images/53405510/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-o/004.jpg</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>53405515</t>
+          <t>BN-GC-19-vin-kr</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/53405515/001.jpg,https://oleks-netizen.github.io/product-images/53405515/002.jpg,https://oleks-netizen.github.io/product-images/53405515/003.jpg,https://oleks-netizen.github.io/product-images/53405515/004.jpg,https://oleks-netizen.github.io/product-images/53405515/005.jpg,https://oleks-netizen.github.io/product-images/53405515/006.jpg,https://oleks-netizen.github.io/product-images/53405515/008.jpg,https://oleks-netizen.github.io/product-images/53405515/009.jpg,https://oleks-netizen.github.io/product-images/53405515/010.jpg,https://oleks-netizen.github.io/product-images/53405515/011.jpg,https://oleks-netizen.github.io/product-images/53405515/012.jpg,https://oleks-netizen.github.io/product-images/53405515/013.jpg,https://oleks-netizen.github.io/product-images/53405515/014.jpg,https://oleks-netizen.github.io/product-images/53405515/015.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-19-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-19-vin-kr/004.jpg</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>90321510</t>
+          <t>BN-GC-28-choko</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90321510/001.jpg,https://oleks-netizen.github.io/product-images/90321510/002.jpg,https://oleks-netizen.github.io/product-images/90321510/004.jpg,https://oleks-netizen.github.io/product-images/90321510/005.jpg,https://oleks-netizen.github.io/product-images/90321510/006.jpg,https://oleks-netizen.github.io/product-images/90321510/007.jpg,https://oleks-netizen.github.io/product-images/90321510/008.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-choko/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-choko/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-choko/004.jpg</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>90321515</t>
+          <t>BN-GC-28-g</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90321515/001.jpg,https://oleks-netizen.github.io/product-images/90321515/002.jpg,https://oleks-netizen.github.io/product-images/90321515/003.jpg,https://oleks-netizen.github.io/product-images/90321515/004.jpg,https://oleks-netizen.github.io/product-images/90321515/005.jpg,https://oleks-netizen.github.io/product-images/90321515/006.jpg,https://oleks-netizen.github.io/product-images/90321515/007.jpg,https://oleks-netizen.github.io/product-images/90321515/008.jpg,https://oleks-netizen.github.io/product-images/90321515/010.jpg,https://oleks-netizen.github.io/product-images/90321515/011.jpg,https://oleks-netizen.github.io/product-images/90321515/012.jpg,https://oleks-netizen.github.io/product-images/90321515/013.jpg,https://oleks-netizen.github.io/product-images/90321515/014.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-g/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-g/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-g/004.jpg</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>90321714</t>
+          <t>BN-GC-28-k</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://oleks-netizen.github.io/product-images/90321714/001.jpg,https://oleks-netizen.github.io/product-images/90321714/002.jpg,https://oleks-netizen.github.io/product-images/90321714/004.jpg,https://oleks-netizen.github.io/product-images/90321714/005.jpg,https://oleks-netizen.github.io/product-images/90321714/006.jpg,https://oleks-netizen.github.io/product-images/90321714/007.jpg,https://oleks-netizen.github.io/product-images/90321714/008.jpg,https://oleks-netizen.github.io/product-images/90321714/009.jpg,https://oleks-netizen.github.io/product-images/90321714/010.jpg</t>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-k/004.jpg</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BN-GC-28-malachite</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-28-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-28-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BN-GC-7-g-kr</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-g-kr/003.jpg</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BN-GC-7-iz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-iz/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-iz/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-iz/004.jpg</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BN-GC-7-k</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k/005.jpg</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BN-GC-7-k-kr</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-k-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BN-GC-7-malachite</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-malachite/004.jpg</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BN-GC-7-navy-blue</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-navy-blue/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-navy-blue/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-navy-blue/003.jpg</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BN-GC-7-nn</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-nn/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-nn/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-nn/003.jpg</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BN-GC-7-o</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-o/003.jpg</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BN-GC-7-red</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-red/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-red/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-red/003.jpg</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BN-GC-7-tiffany</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-tiffany/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-tiffany/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-tiffany/003.jpg</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BN-GC-7-vin</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-vin/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-vin/003.jpg</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BN-GC-7-vin-kr</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/003.jpg,https://oleks-netizen.github.io/product-images/BN-GC-7-vin-kr/005.jpg</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BN-GC-8-g-kr</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-g-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-8-g-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-8-g-kr/004.jpg</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BN-GC-8-k-kr</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-k-kr/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-8-k-kr/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-8-k-kr/003.jpg</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BN-GC-8-o</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://oleks-netizen.github.io/product-images/BN-GC-8-o/001.jpg,https://oleks-netizen.github.io/product-images/BN-GC-8-o/002.jpg,https://oleks-netizen.github.io/product-images/BN-GC-8-o/003.jpg</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>